<commit_message>
Mark US History 8-2 dashboard complete
</commit_message>
<xml_diff>
--- a/8-2/exports/US History 8-2 - Course Outline.xlsx
+++ b/8-2/exports/US History 8-2 - Course Outline.xlsx
@@ -6126,38 +6126,42 @@
       <c r="A304" s="2"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Page</t>
         </is>
       </c>
       <c r="C304" s="5"/>
-      <c r="D304" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
+      <c r="D304" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20.1 | Semester 2 Final Exam Study Guide</t>
         </is>
       </c>
       <c r="E304" s="6"/>
       <c r="F304" s="6"/>
-      <c r="G304" s="6"/>
+      <c r="G304" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Your teacher will provide the final exam study guide here after the final exam is confirmed in Mastery Connect. The study guide should be shorter and targeted to the final exam topics.</t>
+        </is>
+      </c>
       <c r="H304" s="2"/>
     </row>
     <row r="305">
       <c r="A305" s="2"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resource</t>
+          <t xml:space="preserve">Page</t>
         </is>
       </c>
       <c r="C305" s="5"/>
       <c r="D305" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Printable study guide Word document</t>
+          <t xml:space="preserve">20.2 | Semester 2 Final Exam</t>
         </is>
       </c>
       <c r="E305" s="6"/>
       <c r="F305" s="6"/>
       <c r="G305" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">US History 8-2 module JSON files 1-19; build tracker; textbook Topic 5 through Topic 9 pages; Mastery Connect final exam when available</t>
+          <t xml:space="preserve">Your teacher will tell you when and where to complete the Semester 2 Final Exam.</t>
         </is>
       </c>
       <c r="H305" s="2"/>
@@ -6166,33 +6170,73 @@
       <c r="A306" s="2"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C306" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
-        </is>
-      </c>
-      <c r="D306" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C306" s="5"/>
+      <c r="D306" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
+        </is>
+      </c>
       <c r="E306" s="6"/>
       <c r="F306" s="6"/>
-      <c r="G306" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Plan now for reviewer website. Build later as a Canvas module with a downloadable study guide and Mastery Connect final exam directions, matching the Semester 1 pattern.</t>
-        </is>
-      </c>
+      <c r="G306" s="6"/>
       <c r="H306" s="2"/>
     </row>
     <row r="307">
       <c r="A307" s="2"/>
-      <c r="B307" s="2"/>
-      <c r="C307" s="2"/>
-      <c r="D307" s="2"/>
-      <c r="E307" s="2"/>
-      <c r="F307" s="2"/>
-      <c r="G307" s="2"/>
+      <c r="B307" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resource</t>
+        </is>
+      </c>
+      <c r="C307" s="5"/>
+      <c r="D307" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable study guide Word document</t>
+        </is>
+      </c>
+      <c r="E307" s="6"/>
+      <c r="F307" s="6"/>
+      <c r="G307" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teacher-provided final exam or Mastery Connect blueprint will drive the final study guide later. The old 8-2 PDF guide was reviewed and judged too long for middle school use.</t>
+        </is>
+      </c>
       <c r="H307" s="2"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="2"/>
+      <c r="B308" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C308" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D308" s="5"/>
+      <c r="E308" s="6"/>
+      <c r="F308" s="6"/>
+      <c r="G308" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module currently contains placeholder directions for the study guide and final exam.</t>
+        </is>
+      </c>
+      <c r="H308" s="2"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="2"/>
+      <c r="B309" s="2"/>
+      <c r="C309" s="2"/>
+      <c r="D309" s="2"/>
+      <c r="E309" s="2"/>
+      <c r="F309" s="2"/>
+      <c r="G309" s="2"/>
+      <c r="H309" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">

</xml_diff>